<commit_message>
sync(workvault): 2026-10-14 12:04 差分 12 件
</commit_message>
<xml_diff>
--- a/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/LNB管理手順書_草案.xlsx
+++ b/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/LNB管理手順書_草案.xlsx
@@ -22,9 +22,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記録と文書管理" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="チェックシート(日次)" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="チェックシート(月次・異常時)" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="要確認事項一覧" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="申し送り(認証情報)" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="引用と部品照合" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="会議課題一覧(一時)" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="要確認事項一覧" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="申し送り(認証情報)" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="引用と部品照合" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'改訂履歴'!$1:$4</definedName>
@@ -40,9 +41,10 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="12">'記録と文書管理'!$1:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="13">'チェックシート(日次)'!$1:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="14">'チェックシート(月次・異常時)'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="15">'要確認事項一覧'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="16">'申し送り(認証情報)'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="17">'引用と部品照合'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="15">'会議課題一覧(一時)'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="16">'要確認事項一覧'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="17">'申し送り(認証情報)'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="18">'引用と部品照合'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -51,7 +53,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -111,11 +113,23 @@
     <font>
       <name val="游ゴシック"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <strike val="1"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <b val="1"/>
       <color rgb="00833C00"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -125,6 +139,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
       </patternFill>
     </fill>
     <fill>
@@ -213,7 +232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -245,13 +264,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -852,12 +875,12 @@
     </row>
     <row r="7"/>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
@@ -937,7 +960,7 @@
     </row>
     <row r="15"/>
     <row r="16" ht="17.5" customHeight="1">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>ここが埋まっていないことが最大の危険。Pana-CIM と Eg-Pro では、バックアップ障害が2件とも「成否を確認する担当が決まっていなかった」ことで長期化している(Eg-Pro のサブサーバー同期は1年以上、nksv523 は6月から暫定運用のまま)。手順書を作るだけでは同じことが起きる。誰がどこで結果を確認し、失敗時に何をするかまで書くこと。</t>
         </is>
@@ -951,7 +974,7 @@
     </row>
     <row r="17"/>
     <row r="18" ht="16.5" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>LNB の運用: DGS を介した手作業。ジョブを消す前に過去ジョブへエクスポートし、必要時にインポートして戻す。取得目的は特定できていない(慣習として続いている)。検討事項: Pana-CIM で一括取得できないか。保存は Pana-CIM で行う。確認担当: 篠原、大塚、茂木。</t>
         </is>
@@ -1052,12 +1075,12 @@
     </row>
     <row r="7"/>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
@@ -1113,7 +1136,7 @@
     </row>
     <row r="13"/>
     <row r="14" ht="17.5" customHeight="1">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>戻せることを確認していないバックアップは、バックアップではない。§8 が埋まったら、戻す試験を一度やってから本章を書く。</t>
         </is>
@@ -1213,7 +1236,7 @@
     </row>
     <row r="7"/>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>要確認</t>
         </is>
@@ -1240,12 +1263,12 @@
     </row>
     <row r="11"/>
     <row r="12" ht="17.5" customHeight="1">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>欄</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>記載</t>
         </is>
@@ -1337,7 +1360,7 @@
     </row>
     <row r="20"/>
     <row r="21" ht="16.5" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="20" t="inlineStr">
         <is>
           <t>会議では、異常時の連絡先と復旧確認の実施条件を確認事項として挙げたまま結論に至っていない。</t>
         </is>
@@ -1365,12 +1388,12 @@
     </row>
     <row r="24"/>
     <row r="25" ht="17.5" customHeight="1">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>欄</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="17" t="inlineStr">
         <is>
           <t>記載</t>
         </is>
@@ -1450,7 +1473,7 @@
     </row>
     <row r="32"/>
     <row r="33" ht="17.5" customHeight="1">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="A33" s="21" t="inlineStr">
         <is>
           <t>自社とベンダーの境界が決まっていないと、異常時に誰も動かない時間が生まれる。</t>
         </is>
@@ -1553,12 +1576,12 @@
     </row>
     <row r="7"/>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
@@ -1652,12 +1675,12 @@
     </row>
     <row r="17"/>
     <row r="18" ht="17.5" customHeight="1">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
@@ -1751,12 +1774,12 @@
     </row>
     <row r="27"/>
     <row r="28" ht="17.5" customHeight="1">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>期日</t>
         </is>
@@ -1788,7 +1811,7 @@
     </row>
     <row r="31"/>
     <row r="32" ht="17.5" customHeight="1">
-      <c r="A32" s="19" t="inlineStr">
+      <c r="A32" s="21" t="inlineStr">
         <is>
           <t>残り日数から逆算すると、聞き取りを先に片付けないと間に合わない。本書の空欄はすべて聞き取りで埋まるもので、文書作成の作業量ではなく聞き取りの段取りが律速。</t>
         </is>
@@ -1890,7 +1913,7 @@
     </row>
     <row r="7"/>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>点検項目が未確定なので、列名は仮である。§6 が埋まった時点で列を確定させる。</t>
         </is>
@@ -1904,7 +1927,7 @@
     </row>
     <row r="9"/>
     <row r="10" ht="31" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>対象システム</t>
         </is>
@@ -1916,7 +1939,7 @@
       </c>
     </row>
     <row r="11" ht="17.5" customHeight="1">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>年月</t>
         </is>
@@ -1928,7 +1951,7 @@
       </c>
     </row>
     <row r="12" ht="17.5" customHeight="1">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>実施者</t>
         </is>
@@ -1941,37 +1964,37 @@
     </row>
     <row r="13"/>
     <row r="14" ht="17.5" customHeight="1">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>L1</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="17" t="inlineStr">
         <is>
           <t>L2</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>L3</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="17" t="inlineStr">
         <is>
           <t>異常の有無</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="17" t="inlineStr">
         <is>
           <t>実施者</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="17" t="inlineStr">
         <is>
           <t>確認者</t>
         </is>
@@ -2018,7 +2041,7 @@
     </row>
     <row r="18"/>
     <row r="19" ht="16.5" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>ライン別に列を分けてある。接続先が3つあるので、1つにまとめると、どのラインが異常だったのかが残らない。</t>
         </is>
@@ -2046,7 +2069,7 @@
     </row>
     <row r="22"/>
     <row r="23" ht="71.5" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>各ラインの欄</t>
         </is>
@@ -2058,7 +2081,7 @@
       </c>
     </row>
     <row r="24" ht="44.5" customHeight="1">
-      <c r="A24" s="17" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>異常の有無</t>
         </is>
@@ -2070,7 +2093,7 @@
       </c>
     </row>
     <row r="25" ht="71.5" customHeight="1">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>原則</t>
         </is>
@@ -2171,7 +2194,7 @@
     </row>
     <row r="7"/>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>LNB に月次の作業があるかが未確認。枠だけ置く。</t>
         </is>
@@ -2185,27 +2208,27 @@
     </row>
     <row r="9"/>
     <row r="10" ht="17.5" customHeight="1">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>確認項目</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>実施日</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>実施者</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>同席者</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>結果</t>
         </is>
@@ -2235,7 +2258,7 @@
     </row>
     <row r="13"/>
     <row r="14" ht="16.5" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>Pana-CIM と同日に実施する場合は、順序を記録すること。LNB は Pana-CIM のデータを参照しているため、どちらを先に触ったかが後で問題になる。</t>
         </is>
@@ -2263,37 +2286,37 @@
     </row>
     <row r="17"/>
     <row r="18" ht="17.5" customHeight="1">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>時刻</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>ライン</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="17" t="inlineStr">
         <is>
           <t>画面・文言</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="17" t="inlineStr">
         <is>
           <t>接続状態</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="17" t="inlineStr">
         <is>
           <t>中断内容</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="17" t="inlineStr">
         <is>
           <t>連絡先/時刻</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="17" t="inlineStr">
         <is>
           <t>記録No.</t>
         </is>
@@ -2319,7 +2342,7 @@
     </row>
     <row r="21"/>
     <row r="22" ht="16.5" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>画面に出ていた文言をそのまま書く。言い換えると、同じ事象かどうかが後で判定できない。</t>
         </is>
@@ -2347,7 +2370,7 @@
     </row>
     <row r="25"/>
     <row r="26" ht="17.5" customHeight="1">
-      <c r="A26" s="19" t="inlineStr">
+      <c r="A26" s="21" t="inlineStr">
         <is>
           <t>いずれも承認が要る。承認者の記入が無い行は、実施していないものとして扱う。</t>
         </is>
@@ -2361,32 +2384,32 @@
     </row>
     <row r="27"/>
     <row r="28" ht="17.5" customHeight="1">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>実施日</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="17" t="inlineStr">
         <is>
           <t>対象ライン</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="17" t="inlineStr">
         <is>
           <t>承認者</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="17" t="inlineStr">
         <is>
           <t>実施者</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="17" t="inlineStr">
         <is>
           <t>結果・記録No.</t>
         </is>
@@ -2444,7 +2467,7 @@
     </row>
     <row r="34"/>
     <row r="35" ht="16.5" customHeight="1">
-      <c r="A35" s="18" t="inlineStr">
+      <c r="A35" s="20" t="inlineStr">
         <is>
           <t>点検文書ではないが、§14 を消していくための欄として内包する。聞き取りは一度で終わらない。誰にいつ何を聞いたかが残っていないと、同じことを二度聞くか、聞いたつもりで抜ける。</t>
         </is>
@@ -2458,27 +2481,27 @@
     </row>
     <row r="36"/>
     <row r="37" ht="17.5" customHeight="1">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>確認した欄</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="17" t="inlineStr">
         <is>
           <t>確認先</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="17" t="inlineStr">
         <is>
           <t>確認日</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="17" t="inlineStr">
         <is>
           <t>確認した内容</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="17" t="inlineStr">
         <is>
           <t>記入者</t>
         </is>
@@ -2524,7 +2547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2574,14 +2597,14 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>要確認事項一覧</t>
+          <t>会議課題一覧(一時)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>14. 要確認事項一覧</t>
+          <t>会議で上がった課題の一覧(一時掲載)</t>
         </is>
       </c>
       <c r="B6" s="15" t="n"/>
@@ -2593,9 +2616,9 @@
     </row>
     <row r="7"/>
     <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>記入シートの M(未充足一覧)と対応する。埋まったらシート側にも日付を入れる。</t>
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>本シートは会議の場での一覧性を確保するための一時掲載。正本は各管理書(md)の該当章であり、解決後は正本側を更新する。達成度の目安: 反映済み=文書に入った(実機確認や決定が残る)/草案あり=持ち寄り案・骨格まで作成済み(会議の判断で確定)/着手=一部作成/未着手・未決=作業または決定がまだ。</t>
         </is>
       </c>
       <c r="B8" s="15" t="n"/>
@@ -2606,23 +2629,759 @@
       <c r="G8" s="16" t="n"/>
     </row>
     <row r="9"/>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>A. 9-30 会議で挙がった課題12件の達成度</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="16" t="n"/>
+    </row>
+    <row r="11"/>
+    <row r="12" ht="17.5" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>課題</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>達成度</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>現状と残務</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>月次再起動手順</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>反映済み</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>管理書 §7 に実手順ベースで記載(SMT点検日の朝・Pana-CIM停止確認)。チェックシートに月次必須項目あり。残務: LNB 側は月次作業の有無自体が未確認(LNB管理書 §14 No.27)。確認方法: 篠原が現行実施者に聞き取り</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="44.5" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>draw.io 相関図 第一層</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>草案あり</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>会議要件どおりの作り直し案を完成(箱6+境界2・線4本)。既存 drawio は業務フロー図のため第一層には使わない。残務: 会議で DGS の位置づけと各箱の管理担当を確定</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44.5" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>バックアップ(周期・保存)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>反映済み</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>管理書 §8 に「周期は毎日・DGSで取得し Pana-CIM で保存」を明記。日次点検 Step 2 で成否確認。残務: 成否の確認者が未決(§8 で最も重要)。戻す試験は未実施(⑫)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="44.5" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>トラブルシューティング</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>反映済み</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>管理書 §10-1 に事象2件(アンドン異常/稼働モニタ異常(Power BI))→再起動手順、正常画面(TrueCase)併記の方針を追記。残務: 画像14枚のうち13枚の対応付け、色定義、記録フォームの所在</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="44.5" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>チェックシートの有無</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>草案あり</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>「あり」で確定(管理手順書に内包)。三項目(稼働状態/バックアップ結果/保存領域)の判定基準案を作成済み。残務: しきい値を実機画面で決定。記録の確認者</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="58" customHeight="1">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>LNB の点検項目</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>LNB管理書 §6 は枠のみ。公式資料に書かれた「LNB接続状態」を聞き取りの出発点として Step 1 に準備済み。項目名すら定まっていない(会議記録 §7)。聞き取りは篠原が実施。本会議で日程を決めること(ネック)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="58" customHeight="1">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>⑦</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>バックアップのデータ確認(誰が・いつ・どこに)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>L1/L2/L3 それぞれで取得していることは会議で確認済み(会議記録 §5)。各ラインで誰が・いつ・どこに保存しているかが必要。確認の材料として LNB_Collector による現場収集(§5)を準備済み。確認先の候補挙げは篠原が実施</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44.5" customHeight="1">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>⑧</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>LNB と DGS の中身の確認・関連性整理</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>DGS は管理書 §3 用語で「位置づけは要確認」のまま。相関図草案(箱6)でも DGS の管理範囲は「要確認(境界候補)」。調査・整理は篠原が実施し、判定は本会議で。相関図②確定の前提</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="44.5" customHeight="1">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>⑨</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>異常時の連絡先と停止判断者</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>未決</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>役割の行は管理書 §5/LNB管理書 §5 にあり、停止判断者の担当は確定済みだが氏名が空欄。管理責任者の記入待ち(会議記録 §10「本人が担当。後日記入」)。文書側の受け皿は完成済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="31" customHeight="1">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>⑩</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>管理手順書の草案作成</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>着手</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Pana-CIM v0.11(骨格完成)/LNB v0.9(骨格のみ)。残務: v0.5 相当(基準反映版)は11月中</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="58" customHeight="1">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>⑪</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>認証情報の保管先</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>未決</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>LNB 接続 URL 3件に利用者名とパスワードが平文で埋め込まれていることを確認(LNB管理書 §15)。本文に書かない方針は確定済みだが、書かない前提の「安全な保管先」が存在しないため、§4-2・§15 の参照先が決められない</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>⑫</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>復旧(戻す試験)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>未実施</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>管理書 §9 は実施条件・頻度とも要確認のまま。取得できていても戻せるかは別であり(管理書 §9)、試験をしないとバックアップの有効性が未証明。実施条件と頻度の案を持ち寄り済み。本会議で確定すること</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>B. 10-14 会議(13:10)で決定を求める9点</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="n"/>
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="15" t="n"/>
+      <c r="E26" s="15" t="n"/>
+      <c r="F26" s="15" t="n"/>
+      <c r="G26" s="16" t="n"/>
+    </row>
+    <row r="27"/>
+    <row r="28" ht="17.5" customHeight="1">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>決定事項</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>内容と背景</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="31" customHeight="1">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>実機確認の日程</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>最優先。しきい値(正常画面名・色定義・遡り日数・容量)、画像13枚の対応付け、バックアップ保存先の実物確認を1回の訪問で済ませたい</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="17.5" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>LNB 聞き取りの担当と日程</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>最優先。全体のネック。ここが進まないと LNB 管理書は空白のままで、12月の登録に間に合わない</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="17.5" customHeight="1">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>バックアップ成否の確認者</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>管理書 §8 で最も重要</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="17.5" customHeight="1">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>異常時の連絡先と停止判断者の氏名記入</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>文書側の受け皿は完成済み。管理責任者の記入待ち</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="17.5" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>認証情報の保管先</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>保管先を決めれば文書側は記載できる。現状は LNB 接続 URL に平文埋め込み</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="17.5" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>復旧(戻す試験)の実施条件と頻度</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>案を持ち寄り済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="17.5" customHeight="1">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Windows 更新後の扱い</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>RPA 機と同じ「更新の翌日に再起動」にするか</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="17.5" customHeight="1">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>随時再起動の記入欄の可否</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>チェックシートへの記入欄を追加できるか</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="17.5" customHeight="1">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>LNB と DGS の中身確認の担当</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>持ち帰りタスクで未定になっている分。相関図確定の前提</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>C. 解決済みの項目(取り消し線で残す運用の掲載分)</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="n"/>
+      <c r="C39" s="15" t="n"/>
+      <c r="D39" s="15" t="n"/>
+      <c r="E39" s="15" t="n"/>
+      <c r="F39" s="15" t="n"/>
+      <c r="G39" s="16" t="n"/>
+    </row>
+    <row r="40"/>
+    <row r="41" ht="17.5" customHeight="1">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>書</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>解決日と内容</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="31" customHeight="1">
+      <c r="A42" s="18" t="inlineStr">
+        <is>
+          <t>Pana-CIM</t>
+        </is>
+      </c>
+      <c r="B42" s="18" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="C42" s="18" t="inlineStr">
+        <is>
+          <t>CIMC-SV の位置づけ</t>
+        </is>
+      </c>
+      <c r="D42" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-05 解決。VMware 上の仮想マシン(RHEL 6・64ビット)。ESXiホスト 172.25.253.45 上で動く。CIM-A PC・CIM-C PC は物理PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="44.5" customHeight="1">
+      <c r="A43" s="18" t="inlineStr">
+        <is>
+          <t>Pana-CIM</t>
+        </is>
+      </c>
+      <c r="B43" s="18" t="inlineStr">
+        <is>
+          <t>No.1(一部)</t>
+        </is>
+      </c>
+      <c r="C43" s="18" t="inlineStr">
+        <is>
+          <t>再起動手順の原本</t>
+        </is>
+      </c>
+      <c r="D43" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-13 解決。操作手順書 0494-912039(06)「PanaCIM」シートに異常時再起動14手順を確認し、原文との突合で完全性を立証済み(管理書 §10-4 突合表)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="31" customHeight="1">
+      <c r="A44" s="18" t="inlineStr">
+        <is>
+          <t>Pana-CIM</t>
+        </is>
+      </c>
+      <c r="B44" s="18" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="C44" s="18" t="inlineStr">
+        <is>
+          <t>人名・割り当ての確認</t>
+        </is>
+      </c>
+      <c r="D44" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-14 解決。管理責任者＝茂木（由）・倉林、副管理責任者＝石井・茂木（絵）と確定(本人確認)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="44.5" customHeight="1">
+      <c r="A45" s="18" t="inlineStr">
+        <is>
+          <t>LNB</t>
+        </is>
+      </c>
+      <c r="B45" s="18" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="C45" s="18" t="inlineStr">
+        <is>
+          <t>稼働率フォルダの中身の確認</t>
+        </is>
+      </c>
+      <c r="D45" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-14 解決。稼働率フォルダにはラインごとの稼働率データ(Pana-CIM 出力の HTML・20260814-1L.htm)が保存されていることを実物で確認。大塚さんへの確認依頼は取り下げ</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="17.5" customHeight="1">
+      <c r="A46" s="18" t="inlineStr">
+        <is>
+          <t>LNB</t>
+        </is>
+      </c>
+      <c r="B46" s="18" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="C46" s="18" t="inlineStr">
+        <is>
+          <t>人名・割り当ての確認</t>
+        </is>
+      </c>
+      <c r="D46" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-14 解決。Pana-CIM 側 No.27 と同じ内容(§5)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A10:G10"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>手 順 書</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="n"/>
+      <c r="C1" s="12" t="n"/>
+      <c r="D1" s="12" t="n"/>
+      <c r="E1" s="12" t="n"/>
+      <c r="F1" s="12" t="n"/>
+      <c r="G1" s="12" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>型   名</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>ZZZ-90000(仮)</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>目次へ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>作業内容</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>要確認事項一覧</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>14. 要確認事項一覧</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n"/>
+      <c r="C6" s="15" t="n"/>
+      <c r="D6" s="15" t="n"/>
+      <c r="E6" s="15" t="n"/>
+      <c r="F6" s="15" t="n"/>
+      <c r="G6" s="16" t="n"/>
+    </row>
+    <row r="7"/>
+    <row r="8" ht="16.5" customHeight="1">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>記入シートの M(未充足一覧)と対応する。埋まったらシート側にも日付を入れる。</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n"/>
+      <c r="C8" s="15" t="n"/>
+      <c r="D8" s="15" t="n"/>
+      <c r="E8" s="15" t="n"/>
+      <c r="F8" s="15" t="n"/>
+      <c r="G8" s="16" t="n"/>
+    </row>
+    <row r="9"/>
     <row r="10" ht="17.5" customHeight="1">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>確認先</t>
         </is>
@@ -3243,6 +4002,226 @@
       <c r="D39" t="inlineStr">
         <is>
           <t>現行実施者、ベンダー</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="44.5" customHeight="1">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>再起動2種の使い分け</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2026-10-14 実機確認で、LWS の再起動ページに「LNB再起動」「LNB-PC電源OFF」「LNB-PCリブート」の3ボタンがあることを確認。再起動としての2種の対応付け(LNB再起動＝LNBシステム／LNB-PCリブート＝PC自体)はボタン名からの推定【要確認】。実施条件・手順・影響範囲・どちらを選ぶかの判断基準は未確定(§7-1)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>現行実施者、ベンダー</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="31" customHeight="1">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>設定情報の自動バックアップの有効化</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2026-10-14 実機確認で機能の存在を確認。ただし現在は実行されていない。有効化するか、DGS 経由の手作業に寄せるかを決める(§8)。有効化する場合は成否の確認者を同時に決める</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>管理責任者、ベンダー</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="44.5" customHeight="1">
+      <c r="A42" s="18" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B42" s="18" t="inlineStr">
+        <is>
+          <t>稼働率フォルダの中身の確認</t>
+        </is>
+      </c>
+      <c r="C42" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-14 解決。稼働率フォルダには、ラインごとの稼働率データ(Pana-CIM 出力の HTML・20260814-1L.htm)が保存されていることを実物で確認。期間・ロット一覧・仕損率[PPM]・1〜7台目の稼働情報(稼働率・稼働時間・総停止時間)を含む。LNB 側に残せない情報を外部保存している実態とみなせる(§8)。残る確認は保存作業の実施者と自動/手動の別(§8 明細表)</t>
+        </is>
+      </c>
+      <c r="D42" s="18" t="inlineStr">
+        <is>
+          <t>実物確認(篠原)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="17.5" customHeight="1">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Pana-CIM のバックアップ</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Pana-CIM のバックアップは調査段階にあり、不明な状態。管理書(Pana-CIM 側)§8 とあわせて進める</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>作成チーム、現行実施者</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="31" customHeight="1">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>L1 生産設備構成の L2/L3 版</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>LWS の LNB構成情報画面で L1 は確認済み(L1NPM-1〜7・SP70-1)。L2/L3 の同画面は未確認。各ラインの設備一覧・IP・バージョンを確認する(§4-3a)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>現行実施者</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="31" customHeight="1">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>生産設備番号と IP の対応</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>L1 では番号と IP の末尾が一致しない(番号1＝192.168.21.244 等)。対応表を正式な資料として確定するか、画面で都度確認するかを決める(§4-3a)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>現行実施者</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="31" customHeight="1">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>基板バーコードスキャナの赤表示</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>L1 の Pingチェックで 192.168.0.1 の3項目が赤表示(2026-10-14 撮影時点)。赤が異常を意味するか、恒常的な状態か。赤のまま運用してよいか</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>現行実施者</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="17.5" customHeight="1">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>LNB-PC電源OFFの扱い</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>LWS に「LNB-PC電源OFF」ボタンが存在。押してよい場面・押してはいけない場面、実行後の起動手順を確定する(§7-1)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>現行実施者、ベンダー</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="17.5" customHeight="1">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>LWS の認証ID</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>LNB構成情報画面に「認証ID」の表示がある。値は本書に書かない(§15 と同じ扱い)。管理方法の確定は §15 とあわせて行う</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>管理責任者</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="44.5" customHeight="1">
+      <c r="A49" s="18" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>人名・割り当ての確認</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-14 解決。同名は茂木（絵）＝絵美さん（当グループ・スケジュール管理担当）／茂木（由）＝由美子さん（相手グループ）。管理責任者＝茂木（由）・倉林、副管理責任者＝石井・茂木（絵）と確定（§5）。会議記録 §12 の「副管理責任者を倉林さんとし」は本確定と食い違うため、本確定を正とする</t>
+        </is>
+      </c>
+      <c r="D49" s="18" t="inlineStr">
+        <is>
+          <t>篠原のグループによる本人確認</t>
         </is>
       </c>
     </row>
@@ -3259,7 +4238,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3334,7 +4313,7 @@
     </row>
     <row r="7"/>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>本書の作成中に、放置できない状態が見つかった。LNB の接続用ショートカット3件に、利用者名とパスワードが URL のクエリとして平文で埋め込まれている。置き場は 11_USBミラー_E/buckup/15575/desktop/ の L1_LNB.url L2_LNB.url L3_LNB.url。値は本書に書かない。</t>
         </is>
@@ -3348,12 +4327,12 @@
     </row>
     <row r="9"/>
     <row r="10" ht="17.5" customHeight="1">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>事実</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>なぜ問題か</t>
         </is>
@@ -3423,7 +4402,7 @@
     </row>
     <row r="17"/>
     <row r="18" ht="17.5" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3435,7 +4414,7 @@
       </c>
     </row>
     <row r="19" ht="17.5" customHeight="1">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -3447,7 +4426,7 @@
       </c>
     </row>
     <row r="20" ht="17.5" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -3459,7 +4438,7 @@
       </c>
     </row>
     <row r="21" ht="17.5" customHeight="1">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -3472,7 +4451,7 @@
     </row>
     <row r="22"/>
     <row r="23" ht="16.5" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>こちらの判断で消していない。現物を消すと、現場でその経路しか知らない人が入れなくなる可能性がある。rules.md の削除は承認が必要という扱いにも合わせた。</t>
         </is>
@@ -3499,7 +4478,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3574,7 +4553,7 @@
     </row>
     <row r="7"/>
     <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>点検項目ではない。設定の前提として記録しておく。公式資料の記載(付録A-2): 無線スキャナーで部品照合機能を使用するには、LNB設定の部品照合設定を行う必要があります。</t>
         </is>
@@ -3588,7 +4567,7 @@
     </row>
     <row r="9"/>
     <row r="10" ht="17.5" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>未確認</t>
         </is>
@@ -3615,7 +4594,7 @@
     </row>
     <row r="13"/>
     <row r="14" ht="16.5" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>改変せずに載せる。本文は読みやすさのために整えてあるので、食い違いがあれば本付録を正とする。</t>
         </is>
@@ -3643,7 +4622,7 @@
     </row>
     <row r="17"/>
     <row r="18" ht="17.5" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>原文</t>
         </is>
@@ -3670,7 +4649,7 @@
     </row>
     <row r="21"/>
     <row r="22" ht="17.5" customHeight="1">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>原文</t>
         </is>
@@ -3683,7 +4662,7 @@
     </row>
     <row r="23"/>
     <row r="24" ht="16.5" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>上記は製品資料の引用であり、自社 L1〜L3 への適用、設定状態、点検項目を確定するものではない。</t>
         </is>
@@ -3711,7 +4690,7 @@
     </row>
     <row r="27"/>
     <row r="28" ht="17.5" customHeight="1">
-      <c r="A28" s="17" t="inlineStr">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>原文</t>
         </is>
@@ -3723,7 +4702,7 @@
       </c>
     </row>
     <row r="29" ht="17.5" customHeight="1">
-      <c r="A29" s="17" t="inlineStr">
+      <c r="A29" s="19" t="inlineStr">
         <is>
           <t>限界</t>
         </is>
@@ -3750,7 +4729,7 @@
     </row>
     <row r="32"/>
     <row r="33" ht="17.5" customHeight="1">
-      <c r="A33" s="17" t="inlineStr">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>確認したもの</t>
         </is>
@@ -3762,7 +4741,7 @@
       </c>
     </row>
     <row r="34" ht="17.5" customHeight="1">
-      <c r="A34" s="17" t="inlineStr">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>原則</t>
         </is>
@@ -3774,7 +4753,7 @@
       </c>
     </row>
     <row r="35" ht="17.5" customHeight="1">
-      <c r="A35" s="17" t="inlineStr">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>確認できていないもの</t>
         </is>
@@ -3811,7 +4790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4008,7 +4987,7 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>要確認事項一覧</t>
+          <t>会議課題一覧(一時)</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4999,7 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>申し送り(認証情報)</t>
+          <t>要確認事項一覧</t>
         </is>
       </c>
     </row>
@@ -4031,6 +5010,18 @@
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>申し送り(認証情報)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>16.</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>引用と部品照合</t>
         </is>
@@ -4053,6 +5044,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4133,27 +5125,27 @@
     </row>
     <row r="7"/>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>版</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>日付</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>改訂内容</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="17" t="inlineStr">
         <is>
           <t>作成</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>承認</t>
         </is>
@@ -4295,27 +5287,27 @@
       </c>
     </row>
     <row r="14" ht="44.5" customHeight="1">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>0.6</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>人名・割り当てを本人確認により確定。§5 を改訂（管理責任者＝茂木（由）・倉林の2名体制、副管理責任者＝石井・茂木（絵））。茂木（絵）のスケジュール管理担当を明記。§14 No.39 解決</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>篠原</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="18" t="inlineStr">
         <is>
           <t>未</t>
         </is>
@@ -4349,54 +5341,54 @@
       </c>
     </row>
     <row r="16" ht="44.5" customHeight="1">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>0.8</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>稼働率フォルダの中身を実物（20260814-1L.htm）で確認。ラインごとの稼働率データ（期間・ロット一覧・仕損率・1〜7台目の稼働情報）であることを確定し、「LNB では保持できない情報」の根拠に据えた。大塚さんへの確認依頼を取り下げ（§14 No.32 解決）</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>篠原</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
         <is>
           <t>未</t>
         </is>
       </c>
     </row>
     <row r="17" ht="44.5" customHeight="1">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>0.9</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>報告準備。§4-4 に図の読み方（種別ラベル・凡例）と PLM 閲覧問題の現状（大塚さん対応中・解決後に図解を拡充）を追記。構成図に種別ラベル・凡例・稼働率フォルダ（実物確認済み）を反映し視認性を改善</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="18" t="inlineStr">
         <is>
           <t>篠原</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="18" t="inlineStr">
         <is>
           <t>未</t>
         </is>
@@ -4489,7 +5481,7 @@
     </row>
     <row r="7"/>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
@@ -4516,7 +5508,7 @@
     </row>
     <row r="11"/>
     <row r="12" ht="17.5" customHeight="1">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>対象</t>
         </is>
@@ -4528,7 +5520,7 @@
       </c>
     </row>
     <row r="13" ht="17.5" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>分冊</t>
         </is>
@@ -4540,7 +5532,7 @@
       </c>
     </row>
     <row r="14" ht="17.5" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>分担</t>
         </is>
@@ -4552,7 +5544,7 @@
       </c>
     </row>
     <row r="15" ht="17.5" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>環境</t>
         </is>
@@ -4564,7 +5556,7 @@
       </c>
     </row>
     <row r="16" ht="17.5" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>未検証</t>
         </is>
@@ -4591,7 +5583,7 @@
     </row>
     <row r="19"/>
     <row r="20" ht="16.5" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>詳細は「LNB・Pana-CIM_管理文書作成_会議記録_追補.md」を参照。本章には経緯の詳細を書かない。</t>
         </is>
@@ -4605,7 +5597,7 @@
     </row>
     <row r="21"/>
     <row r="22" ht="17.5" customHeight="1">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>経緯</t>
         </is>
@@ -4617,7 +5609,7 @@
       </c>
     </row>
     <row r="23" ht="17.5" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>教訓</t>
         </is>
@@ -4630,7 +5622,7 @@
     </row>
     <row r="24"/>
     <row r="25" ht="16.5" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>本書は LNB_点検文書_情報記入シート.md の記入済み範囲だけで組んだ草案である。同シートの F(点検項目)は全行が空欄。点検の基準を推測で埋めていない。判定基準を創作すると、異常を正常と読む文書になる。</t>
         </is>
@@ -4733,12 +5725,12 @@
     </row>
     <row r="7"/>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>語</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>意味</t>
         </is>
@@ -4951,12 +5943,12 @@
     </row>
     <row r="7"/>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
@@ -5062,7 +6054,7 @@
     </row>
     <row r="18"/>
     <row r="19" ht="16.5" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>保管庫内の資料から確認できた範囲。11_USBミラー_E に残っていたデスクトップのショートカット3件(L1_LNB.url L2_LNB.url L3_LNB.url)から読み取った。</t>
         </is>
@@ -5076,17 +6068,17 @@
     </row>
     <row r="20"/>
     <row r="21" ht="17.5" customHeight="1">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>ライン</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>接続先</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>画面</t>
         </is>
@@ -5145,7 +6137,7 @@
     </row>
     <row r="25"/>
     <row r="26" ht="16.5" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>第4オクテットが 11/21/31 と並んでおり、ラインごとに10ずつ繰り上がる付番と見える。L4以降が存在するかは要確認。</t>
         </is>
@@ -5159,12 +6151,12 @@
     </row>
     <row r="27"/>
     <row r="28" ht="17.5" customHeight="1">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
@@ -5258,7 +6250,7 @@
     </row>
     <row r="37"/>
     <row r="38" ht="31" customHeight="1">
-      <c r="A38" s="17" t="inlineStr">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>参照</t>
         </is>
@@ -5270,7 +6262,7 @@
       </c>
     </row>
     <row r="39" ht="31" customHeight="1">
-      <c r="A39" s="17" t="inlineStr">
+      <c r="A39" s="19" t="inlineStr">
         <is>
           <t>更新方針</t>
         </is>
@@ -5372,17 +6364,17 @@
     </row>
     <row r="7"/>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>役割</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>氏名</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>不在時の代行</t>
         </is>
@@ -5509,7 +6501,7 @@
     </row>
     <row r="16"/>
     <row r="17" ht="16.5" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>人名と割り当ては 2026-10-14、篠原のグループによる本人確認で確定。会議記録 §12 の「副管理責任者を倉林さんとし」は本確認と食い違うため、本確認を正とする。</t>
         </is>
@@ -5537,7 +6529,7 @@
     </row>
     <row r="20"/>
     <row r="21" ht="31" customHeight="1">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>環境</t>
         </is>
@@ -5549,7 +6541,7 @@
       </c>
     </row>
     <row r="22" ht="17.5" customHeight="1">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>原則</t>
         </is>
@@ -5649,7 +6641,7 @@
     </row>
     <row r="7"/>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>点検項目が未確定のため、本章は枠のみである。会議資料にも引き継ぎ資料にも LNB の点検項目の記載がなく、現行実施者への聞き取りが済むまで本体は書けない。実施してよい時間帯、所要時間の目安、休日の実施有無はいずれも要確認。</t>
         </is>
@@ -5677,7 +6669,7 @@
     </row>
     <row r="11"/>
     <row r="12" ht="16.5" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>聞き取りの結果をこの形で埋める。各項目を Step として並べ、1項目ごとに次の6点を書く。</t>
         </is>
@@ -5691,12 +6683,12 @@
     </row>
     <row r="13"/>
     <row r="14" ht="17.5" customHeight="1">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>書く欄</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>書き方</t>
         </is>
@@ -5790,7 +6782,7 @@
     </row>
     <row r="23"/>
     <row r="24" ht="17.5" customHeight="1">
-      <c r="A24" s="17" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>理由</t>
         </is>
@@ -5802,7 +6794,7 @@
       </c>
     </row>
     <row r="25" ht="17.5" customHeight="1">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>進め方</t>
         </is>
@@ -5829,7 +6821,7 @@
     </row>
     <row r="28"/>
     <row r="29" ht="17.5" customHeight="1">
-      <c r="A29" s="19" t="inlineStr">
+      <c r="A29" s="21" t="inlineStr">
         <is>
           <t>確定した点検項目ではない。公式資料に「表示される」と書かれている項目なので、聞き取りの出発点として置く。</t>
         </is>
@@ -5843,12 +6835,12 @@
     </row>
     <row r="30"/>
     <row r="31" ht="17.5" customHeight="1">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
@@ -5916,7 +6908,7 @@
     </row>
     <row r="37"/>
     <row r="38" ht="16.5" customHeight="1">
-      <c r="A38" s="18" t="inlineStr">
+      <c r="A38" s="20" t="inlineStr">
         <is>
           <t>判定基準が決まるまでは、見たものをそのまま書く。○×で記録を始めると、基準を決めたあとに過去の記録が読めなくなる。</t>
         </is>
@@ -5944,7 +6936,7 @@
     </row>
     <row r="41"/>
     <row r="42" ht="17.5" customHeight="1">
-      <c r="A42" s="17" t="inlineStr">
+      <c r="A42" s="19" t="inlineStr">
         <is>
           <t>方針</t>
         </is>
@@ -6050,7 +7042,7 @@
     </row>
     <row r="7"/>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>頻度区分</t>
         </is>
@@ -6062,7 +7054,7 @@
       </c>
     </row>
     <row r="9" ht="17.5" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>月次の有無</t>
         </is>
@@ -6074,7 +7066,7 @@
       </c>
     </row>
     <row r="10" ht="17.5" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>順序の制約</t>
         </is>
@@ -6101,7 +7093,7 @@
     </row>
     <row r="13"/>
     <row r="14" ht="17.5" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -6113,7 +7105,7 @@
       </c>
     </row>
     <row r="15" ht="17.5" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -6125,7 +7117,7 @@
       </c>
     </row>
     <row r="16" ht="17.5" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -6137,7 +7129,7 @@
       </c>
     </row>
     <row r="17" ht="17.5" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>4</t>
         </is>

</xml_diff>

<commit_message>
sync(workvault): 2026-10-14 12:12 差分 8 件
</commit_message>
<xml_diff>
--- a/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/LNB管理手順書_草案.xlsx
+++ b/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/LNB管理手順書_草案.xlsx
@@ -2322,7 +2322,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="17.5" customHeight="1">
+    <row r="19" ht="24" customHeight="1">
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
@@ -2331,7 +2331,7 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
     </row>
-    <row r="20" ht="17.5" customHeight="1">
+    <row r="20" ht="24" customHeight="1">
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
@@ -2507,14 +2507,14 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="17.5" customHeight="1">
+    <row r="38" ht="24" customHeight="1">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
     </row>
-    <row r="39" ht="17.5" customHeight="1">
+    <row r="39" ht="24" customHeight="1">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>

</xml_diff>

<commit_message>
sync(workvault): 2026-10-14 14:34 差分 9 件
</commit_message>
<xml_diff>
--- a/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/LNB管理手順書_草案.xlsx
+++ b/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/LNB管理手順書_草案.xlsx
@@ -695,7 +695,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>0.9(草案・未検証)</t>
+          <t>0.11(草案・未検証)</t>
         </is>
       </c>
     </row>
@@ -5056,7 +5056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5389,6 +5389,60 @@
         </is>
       </c>
       <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>未</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="44.5" customHeight="1">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>0.10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>用語の正式名称を確定（§3）。LNB＝Line Network Box の略（実装設備群と NPM-DGS を接続する中継・ライン管理システム）、DGS＝NPM-DGS（Data Generation System）。LWS 画面タイトルとの整合を明記</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>篠原</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>未</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="31" customHeight="1">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>0.11</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>§3 の LNB 正式名称の出典を訂正。「ユーザー本人の確認」→「竹渕さんのチャット情報」。内容の変更なし（出典の記載のみ）</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>篠原</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>未</t>
         </is>
@@ -5736,7 +5790,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="17.5" customHeight="1">
+    <row r="9" ht="31" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>LNB</t>
@@ -5744,7 +5798,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>社内での呼び名。本書では、承認済みの L1〜L3 端末と、そこで稼働する LNB ソフトを対象とする。iLNB と同一であるとは断定しない</t>
+          <t>Line Network Box の略。実装設備群と NPM-DGS（Data Generation System）を接続する中継・ライン管理システム（2026-10-14、竹渕さんのチャット情報により確定）。本書では、承認済みの L1〜L3 端末と、そこで稼働する LNB ソフトを対象とする。iLNB と同一であるとは断定しない</t>
         </is>
       </c>
     </row>
@@ -5768,7 +5822,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LNB の画面を提供しているアプリケーションの経路名。接続先URLの /lws/ にあたる。正式な呼称は要確認</t>
+          <t>LNB の画面を提供しているアプリケーションの経路名。接続先URLの /lws/ にあたる。画面タイトル「Line Network Box」は LNB の正式名称確定と整合。正式な呼称は要確認</t>
         </is>
       </c>
     </row>
@@ -5820,7 +5874,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="17.5" customHeight="1">
+    <row r="16" ht="31" customHeight="1">
       <c r="A16" t="inlineStr">
         <is>
           <t>DGS</t>
@@ -5828,7 +5882,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>LNB のバックアップ経路に現れる系。本書での位置づけは要確認</t>
+          <t>NPM-DGS（Data Generation System）。実装データを生成・管理する上位システム。LNB のバックアップ経路に現れる。LWS の Pingチェック画面では「上位システム」として表示（IP 172.25.253.10）。本書での位置づけは要確認</t>
         </is>
       </c>
     </row>

</xml_diff>